<commit_message>
fix: update date formatting in Excel exporter and corresponding tests for consistency
</commit_message>
<xml_diff>
--- a/mongo_exports/biblioteca_normalizada.xlsx
+++ b/mongo_exports/biblioteca_normalizada.xlsx
@@ -21,11 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -58,12 +54,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -475,8 +469,10 @@
           <t>El Aleph - Ed 322</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>19792</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>09/03/1954</t>
+        </is>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -526,8 +522,10 @@
           <t>La casa de los espíritus - Ed 624</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>31773</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>27/12/1986</t>
+        </is>
       </c>
       <c r="D5" t="n">
         <v>2</v>
@@ -561,8 +559,10 @@
           <t>Crónica de una muerte anunciada - Ed 780</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>36917</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>26/01/2001</t>
+        </is>
       </c>
       <c r="D7" t="n">
         <v>6</v>
@@ -580,8 +580,10 @@
           <t>Crónica de una muerte anunciada - Ed 269</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
-        <v>37818</v>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>16/07/2003</t>
+        </is>
       </c>
       <c r="D8" t="n">
         <v>6</v>
@@ -615,8 +617,10 @@
           <t>Ficciones - Ed 844</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
-        <v>29698</v>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>22/04/1981</t>
+        </is>
       </c>
       <c r="D10" t="n">
         <v>9</v>
@@ -634,8 +638,10 @@
           <t>Pedro Páramo - Ed 746</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
-        <v>40620</v>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>18/03/2011</t>
+        </is>
       </c>
       <c r="D11" t="n">
         <v>9</v>
@@ -685,8 +691,10 @@
           <t>Rayuela - Ed 76</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
-        <v>35600</v>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>19/06/1997</t>
+        </is>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -736,8 +744,10 @@
           <t>El amor en los tiempos del cólera - Ed 120</t>
         </is>
       </c>
-      <c r="C17" s="2" t="n">
-        <v>30646</v>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>26/11/1983</t>
+        </is>
       </c>
       <c r="D17" t="n">
         <v>16</v>
@@ -851,8 +861,10 @@
           <t>Ficciones - Ed 213</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n">
-        <v>25002</v>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>13/06/1968</t>
+        </is>
       </c>
       <c r="D24" t="n">
         <v>2</v>
@@ -886,8 +898,10 @@
           <t>cien años de soledad - ed 142</t>
         </is>
       </c>
-      <c r="C26" s="2" t="n">
-        <v>23963</v>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>09/08/1965</t>
+        </is>
       </c>
       <c r="D26" t="n">
         <v>1</v>
@@ -905,8 +919,10 @@
           <t>La casa de los espíritus - Ed 901</t>
         </is>
       </c>
-      <c r="C27" s="2" t="n">
-        <v>39210</v>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>08/05/2007</t>
+        </is>
       </c>
       <c r="D27" t="n">
         <v>2</v>
@@ -924,8 +940,10 @@
           <t>El Aleph - Ed 772</t>
         </is>
       </c>
-      <c r="C28" s="2" t="n">
-        <v>27006</v>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>08/12/1973</t>
+        </is>
       </c>
       <c r="D28" t="n">
         <v>2</v>
@@ -959,8 +977,10 @@
           <t>Don Quijote de la Mancha - Ed 67</t>
         </is>
       </c>
-      <c r="C30" s="2" t="n">
-        <v>31027</v>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11/12/1984</t>
+        </is>
       </c>
       <c r="D30" t="n">
         <v>2</v>
@@ -994,8 +1014,10 @@
           <t>Pedro Páramo - Ed 504</t>
         </is>
       </c>
-      <c r="C32" s="2" t="n">
-        <v>39077</v>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>26/12/2006</t>
+        </is>
       </c>
       <c r="D32" t="n">
         <v>31</v>
@@ -1141,8 +1163,10 @@
           <t>Rayuela - Ed 784</t>
         </is>
       </c>
-      <c r="C41" s="2" t="n">
-        <v>37732</v>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>21/04/2003</t>
+        </is>
       </c>
       <c r="D41" t="n">
         <v>6</v>
@@ -1160,8 +1184,10 @@
           <t>El amor en los tiempos del cólera - Ed 185</t>
         </is>
       </c>
-      <c r="C42" s="2" t="n">
-        <v>23668</v>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>18/10/1964</t>
+        </is>
       </c>
       <c r="D42" t="n">
         <v>16</v>
@@ -1227,8 +1253,10 @@
           <t>Crónica de una muerte anunciada - Ed 410</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n">
-        <v>27380</v>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>17/12/1974</t>
+        </is>
       </c>
       <c r="D46" t="n">
         <v>2</v>
@@ -1262,8 +1290,10 @@
           <t>Rayuela - Ed 566</t>
         </is>
       </c>
-      <c r="C48" s="2" t="n">
-        <v>31882</v>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>15/04/1987</t>
+        </is>
       </c>
       <c r="D48" t="n">
         <v>1</v>
@@ -1313,8 +1343,10 @@
           <t>El amor en los tiempos del cólera - Ed 662</t>
         </is>
       </c>
-      <c r="C51" s="2" t="n">
-        <v>22455</v>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>23/06/1961</t>
+        </is>
       </c>
       <c r="D51" t="n">
         <v>31</v>
@@ -1332,8 +1364,10 @@
           <t>Cien años de soledad - Ed 815</t>
         </is>
       </c>
-      <c r="C52" s="2" t="n">
-        <v>30761</v>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>20/03/1984</t>
+        </is>
       </c>
       <c r="D52" t="n">
         <v>16</v>
@@ -1351,8 +1385,10 @@
           <t>Crónica de una muerte anunciada - Ed 623</t>
         </is>
       </c>
-      <c r="C53" s="2" t="n">
-        <v>30325</v>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>09/01/1983</t>
+        </is>
       </c>
       <c r="D53" t="n">
         <v>16</v>
@@ -1434,8 +1470,10 @@
           <t>Ficciones - Ed 433</t>
         </is>
       </c>
-      <c r="C58" s="2" t="n">
-        <v>19568</v>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>28/07/1953</t>
+        </is>
       </c>
       <c r="D58" t="n">
         <v>9</v>
@@ -1485,8 +1523,10 @@
           <t>Pedro Páramo - Ed 881</t>
         </is>
       </c>
-      <c r="C61" s="2" t="n">
-        <v>30443</v>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>07/05/1983</t>
+        </is>
       </c>
       <c r="D61" t="n">
         <v>1</v>
@@ -1504,8 +1544,10 @@
           <t>Crónica de una muerte anunciada - Ed 944</t>
         </is>
       </c>
-      <c r="C62" s="2" t="n">
-        <v>31075</v>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>28/01/1985</t>
+        </is>
       </c>
       <c r="D62" t="n">
         <v>6</v>
@@ -1523,8 +1565,10 @@
           <t>Don Quijote de la Mancha - Ed 923</t>
         </is>
       </c>
-      <c r="C63" s="2" t="n">
-        <v>26115</v>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>01/07/1971</t>
+        </is>
       </c>
       <c r="D63" t="n">
         <v>6</v>
@@ -1558,8 +1602,10 @@
           <t>Pedro Páramo - Ed 25</t>
         </is>
       </c>
-      <c r="C65" s="2" t="n">
-        <v>40418</v>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>28/08/2010</t>
+        </is>
       </c>
       <c r="D65" t="n">
         <v>2</v>
@@ -1641,8 +1687,10 @@
           <t>Don Quijote de la Mancha - Ed 820</t>
         </is>
       </c>
-      <c r="C70" s="2" t="n">
-        <v>20885</v>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>06/03/1957</t>
+        </is>
       </c>
       <c r="D70" t="n">
         <v>2</v>
@@ -1692,8 +1740,10 @@
           <t>La casa de los espíritus - Ed 981</t>
         </is>
       </c>
-      <c r="C73" s="2" t="n">
-        <v>22233</v>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>13/11/1960</t>
+        </is>
       </c>
       <c r="D73" t="n">
         <v>6</v>
@@ -1711,8 +1761,10 @@
           <t>El amor en los tiempos del cólera - Ed 31</t>
         </is>
       </c>
-      <c r="C74" s="2" t="n">
-        <v>39465</v>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>18/01/2008</t>
+        </is>
       </c>
       <c r="D74" t="n">
         <v>6</v>
@@ -1746,8 +1798,10 @@
           <t>Ficciones - Ed 647</t>
         </is>
       </c>
-      <c r="C76" s="2" t="n">
-        <v>45222</v>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>23/10/2023</t>
+        </is>
       </c>
       <c r="D76" t="n">
         <v>2</v>
@@ -1861,8 +1915,10 @@
           <t>La ciudad y los perros - Ed 810</t>
         </is>
       </c>
-      <c r="C83" s="2" t="n">
-        <v>19058</v>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>05/03/1952</t>
+        </is>
       </c>
       <c r="D83" t="n">
         <v>6</v>
@@ -1912,8 +1968,10 @@
           <t>Pedro Páramo - Ed 304</t>
         </is>
       </c>
-      <c r="C86" s="2" t="n">
-        <v>22460</v>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>28/06/1961</t>
+        </is>
       </c>
       <c r="D86" t="n">
         <v>16</v>
@@ -1931,8 +1989,10 @@
           <t>Don Quijote de la Mancha - Ed 149</t>
         </is>
       </c>
-      <c r="C87" s="2" t="n">
-        <v>20531</v>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>17/03/1956</t>
+        </is>
       </c>
       <c r="D87" t="n">
         <v>6</v>
@@ -1950,8 +2010,10 @@
           <t>La ciudad y los perros - Ed 68</t>
         </is>
       </c>
-      <c r="C88" s="2" t="n">
-        <v>43942</v>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>21/04/2020</t>
+        </is>
       </c>
       <c r="D88" t="n">
         <v>6</v>
@@ -1985,8 +2047,10 @@
           <t>Rayuela - Ed 432</t>
         </is>
       </c>
-      <c r="C90" s="2" t="n">
-        <v>32614</v>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>16/04/1989</t>
+        </is>
       </c>
       <c r="D90" t="n">
         <v>31</v>
@@ -2084,8 +2148,10 @@
           <t>Pedro Páramo - Ed 553</t>
         </is>
       </c>
-      <c r="C96" s="2" t="n">
-        <v>37017</v>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>06/05/2001</t>
+        </is>
       </c>
       <c r="D96" t="n">
         <v>9</v>
@@ -2333,7 +2399,7 @@
           <t>María García</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>m.garcia@email.com</t>
         </is>
@@ -2348,7 +2414,7 @@
           <t>Ana Martínez</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>ana.mar_libros@email.com</t>
         </is>
@@ -2363,7 +2429,7 @@
           <t>Juan Pérez</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>juan.perez@email.com</t>
         </is>
@@ -2378,7 +2444,7 @@
           <t>Carlos López</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>clopez_88@email.com</t>
         </is>
@@ -2448,8 +2514,10 @@
       <c r="C2" t="n">
         <v>27</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>46164</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2467,11 +2535,15 @@
       <c r="C3" t="n">
         <v>16</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>46174</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2489,8 +2561,10 @@
       <c r="C4" t="n">
         <v>65</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>45294</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>03/01/2024</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2508,11 +2582,15 @@
       <c r="C5" t="n">
         <v>7</v>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>46174</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -2530,11 +2608,15 @@
       <c r="C6" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>45409</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>45419</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>27/04/2024</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>07/05/2024</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -2552,11 +2634,15 @@
       <c r="C7" t="n">
         <v>88</v>
       </c>
-      <c r="D7" s="2" t="n">
-        <v>45409</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>45419</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>27/04/2024</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>07/05/2024</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -2574,11 +2660,15 @@
       <c r="C8" t="n">
         <v>40</v>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>45311</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>45321</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>20/01/2024</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>30/01/2024</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -2596,11 +2686,15 @@
       <c r="C9" t="n">
         <v>82</v>
       </c>
-      <c r="D9" s="2" t="n">
-        <v>45293</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>45303</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>02/01/2024</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>12/01/2024</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -2618,8 +2712,10 @@
       <c r="C10" t="n">
         <v>82</v>
       </c>
-      <c r="D10" s="2" t="n">
-        <v>46164</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -2637,8 +2733,10 @@
       <c r="C11" t="n">
         <v>41</v>
       </c>
-      <c r="D11" s="2" t="n">
-        <v>45395</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>13/04/2024</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -2656,8 +2754,10 @@
       <c r="C12" t="n">
         <v>61</v>
       </c>
-      <c r="D12" s="2" t="n">
-        <v>46164</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -2675,8 +2775,10 @@
       <c r="C13" t="n">
         <v>86</v>
       </c>
-      <c r="D13" s="2" t="n">
-        <v>45305</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>14/01/2024</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -2694,11 +2796,15 @@
       <c r="C14" t="n">
         <v>14</v>
       </c>
-      <c r="D14" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>46174</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -2716,8 +2822,10 @@
       <c r="C15" t="n">
         <v>22</v>
       </c>
-      <c r="D15" s="2" t="n">
-        <v>45387</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>05/04/2024</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -2735,11 +2843,15 @@
       <c r="C16" t="n">
         <v>43</v>
       </c>
-      <c r="D16" s="2" t="n">
-        <v>45309</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>45319</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>18/01/2024</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>28/01/2024</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -2757,8 +2869,10 @@
       <c r="C17" t="n">
         <v>61</v>
       </c>
-      <c r="D17" s="2" t="n">
-        <v>45393</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>11/04/2024</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -2776,8 +2890,10 @@
       <c r="C18" t="n">
         <v>24</v>
       </c>
-      <c r="D18" s="2" t="n">
-        <v>45376</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>25/03/2024</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -2795,8 +2911,10 @@
       <c r="C19" t="n">
         <v>11</v>
       </c>
-      <c r="D19" s="2" t="n">
-        <v>46164</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -2814,8 +2932,10 @@
       <c r="C20" t="n">
         <v>24</v>
       </c>
-      <c r="D20" s="2" t="n">
-        <v>45409</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>27/04/2024</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -2833,11 +2953,15 @@
       <c r="C21" t="n">
         <v>42</v>
       </c>
-      <c r="D21" s="2" t="n">
-        <v>45296</v>
-      </c>
-      <c r="E21" s="2" t="n">
-        <v>45306</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>05/01/2024</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>15/01/2024</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -2855,11 +2979,15 @@
       <c r="C22" t="n">
         <v>93</v>
       </c>
-      <c r="D22" s="2" t="n">
-        <v>45337</v>
-      </c>
-      <c r="E22" s="2" t="n">
-        <v>45347</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>15/02/2024</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>25/02/2024</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -2877,11 +3005,15 @@
       <c r="C23" t="n">
         <v>8</v>
       </c>
-      <c r="D23" s="2" t="n">
-        <v>45337</v>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>45347</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>15/02/2024</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>25/02/2024</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -2899,8 +3031,10 @@
       <c r="C24" t="n">
         <v>26</v>
       </c>
-      <c r="D24" s="2" t="n">
-        <v>46164</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -2918,8 +3052,10 @@
       <c r="C25" t="n">
         <v>55</v>
       </c>
-      <c r="D25" s="2" t="n">
-        <v>45358</v>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>07/03/2024</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -2937,11 +3073,15 @@
       <c r="C26" t="n">
         <v>89</v>
       </c>
-      <c r="D26" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>46174</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -2959,8 +3099,10 @@
       <c r="C27" t="n">
         <v>8</v>
       </c>
-      <c r="D27" s="2" t="n">
-        <v>45391</v>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>09/04/2024</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -2978,11 +3120,15 @@
       <c r="C28" t="n">
         <v>96</v>
       </c>
-      <c r="D28" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>46174</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -3000,11 +3146,15 @@
       <c r="C29" t="n">
         <v>35</v>
       </c>
-      <c r="D29" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>46174</v>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -3022,8 +3172,10 @@
       <c r="C30" t="n">
         <v>39</v>
       </c>
-      <c r="D30" s="2" t="n">
-        <v>46164</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -3041,11 +3193,15 @@
       <c r="C31" t="n">
         <v>43</v>
       </c>
-      <c r="D31" s="2" t="n">
-        <v>45406</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>45416</v>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>24/04/2024</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>04/05/2024</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -3063,11 +3219,15 @@
       <c r="C32" t="n">
         <v>89</v>
       </c>
-      <c r="D32" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>46174</v>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -3085,11 +3245,15 @@
       <c r="C33" t="n">
         <v>80</v>
       </c>
-      <c r="D33" s="2" t="n">
-        <v>45346</v>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>45356</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>24/02/2024</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>05/03/2024</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -3107,8 +3271,10 @@
       <c r="C34" t="n">
         <v>99</v>
       </c>
-      <c r="D34" s="2" t="n">
-        <v>45410</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>28/04/2024</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -3126,8 +3292,10 @@
       <c r="C35" t="n">
         <v>28</v>
       </c>
-      <c r="D35" s="2" t="n">
-        <v>46164</v>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -3145,11 +3313,15 @@
       <c r="C36" t="n">
         <v>68</v>
       </c>
-      <c r="D36" s="2" t="n">
-        <v>45320</v>
-      </c>
-      <c r="E36" s="2" t="n">
-        <v>45330</v>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>29/01/2024</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>08/02/2024</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -3167,8 +3339,10 @@
       <c r="C37" t="n">
         <v>40</v>
       </c>
-      <c r="D37" s="2" t="n">
-        <v>45392</v>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>10/04/2024</t>
+        </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -3186,8 +3360,10 @@
       <c r="C38" t="n">
         <v>5</v>
       </c>
-      <c r="D38" s="2" t="n">
-        <v>45367</v>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>16/03/2024</t>
+        </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -3205,8 +3381,10 @@
       <c r="C39" t="n">
         <v>95</v>
       </c>
-      <c r="D39" s="2" t="n">
-        <v>45385</v>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>03/04/2024</t>
+        </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -3224,8 +3402,10 @@
       <c r="C40" t="n">
         <v>93</v>
       </c>
-      <c r="D40" s="2" t="n">
-        <v>45300</v>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>09/01/2024</t>
+        </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -3243,8 +3423,10 @@
       <c r="C41" t="n">
         <v>39</v>
       </c>
-      <c r="D41" s="2" t="n">
-        <v>45300</v>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>09/01/2024</t>
+        </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -3262,8 +3444,10 @@
       <c r="C42" t="n">
         <v>9</v>
       </c>
-      <c r="D42" s="2" t="n">
-        <v>45412</v>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>30/04/2024</t>
+        </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -3281,11 +3465,15 @@
       <c r="C43" t="n">
         <v>93</v>
       </c>
-      <c r="D43" s="2" t="n">
-        <v>45328</v>
-      </c>
-      <c r="E43" s="2" t="n">
-        <v>45338</v>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>06/02/2024</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>16/02/2024</t>
+        </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -3303,8 +3491,10 @@
       <c r="C44" t="n">
         <v>1</v>
       </c>
-      <c r="D44" s="2" t="n">
-        <v>45296</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>05/01/2024</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -3322,8 +3512,10 @@
       <c r="C45" t="n">
         <v>30</v>
       </c>
-      <c r="D45" s="2" t="n">
-        <v>45296</v>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>05/01/2024</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -3341,8 +3533,10 @@
       <c r="C46" t="n">
         <v>58</v>
       </c>
-      <c r="D46" s="2" t="n">
-        <v>45384</v>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>02/04/2024</t>
+        </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -3360,8 +3554,10 @@
       <c r="C47" t="n">
         <v>74</v>
       </c>
-      <c r="D47" s="2" t="n">
-        <v>45348</v>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>26/02/2024</t>
+        </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -3379,8 +3575,10 @@
       <c r="C48" t="n">
         <v>33</v>
       </c>
-      <c r="D48" s="2" t="n">
-        <v>45362</v>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>11/03/2024</t>
+        </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -3398,8 +3596,10 @@
       <c r="C49" t="n">
         <v>18</v>
       </c>
-      <c r="D49" s="2" t="n">
-        <v>45362</v>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>11/03/2024</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -3417,8 +3617,10 @@
       <c r="C50" t="n">
         <v>87</v>
       </c>
-      <c r="D50" s="2" t="n">
-        <v>45362</v>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>11/03/2024</t>
+        </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -3436,11 +3638,15 @@
       <c r="C51" t="n">
         <v>72</v>
       </c>
-      <c r="D51" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E51" s="2" t="n">
-        <v>46174</v>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -3458,11 +3664,15 @@
       <c r="C52" t="n">
         <v>35</v>
       </c>
-      <c r="D52" s="2" t="n">
-        <v>45373</v>
-      </c>
-      <c r="E52" s="2" t="n">
-        <v>45383</v>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>22/03/2024</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>01/04/2024</t>
+        </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -3480,11 +3690,15 @@
       <c r="C53" t="n">
         <v>37</v>
       </c>
-      <c r="D53" s="2" t="n">
-        <v>45366</v>
-      </c>
-      <c r="E53" s="2" t="n">
-        <v>45376</v>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>15/03/2024</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>25/03/2024</t>
+        </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -3502,11 +3716,15 @@
       <c r="C54" t="n">
         <v>90</v>
       </c>
-      <c r="D54" s="2" t="n">
-        <v>45366</v>
-      </c>
-      <c r="E54" s="2" t="n">
-        <v>45376</v>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>15/03/2024</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>25/03/2024</t>
+        </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -3524,11 +3742,15 @@
       <c r="C55" t="n">
         <v>48</v>
       </c>
-      <c r="D55" s="2" t="n">
-        <v>45366</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>45376</v>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>15/03/2024</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>25/03/2024</t>
+        </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -3546,8 +3768,10 @@
       <c r="C56" t="n">
         <v>64</v>
       </c>
-      <c r="D56" s="2" t="n">
-        <v>45334</v>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>12/02/2024</t>
+        </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -3565,11 +3789,15 @@
       <c r="C57" t="n">
         <v>3</v>
       </c>
-      <c r="D57" s="2" t="n">
-        <v>45342</v>
-      </c>
-      <c r="E57" s="2" t="n">
-        <v>45352</v>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>20/02/2024</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>01/03/2024</t>
+        </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -3587,11 +3815,15 @@
       <c r="C58" t="n">
         <v>33</v>
       </c>
-      <c r="D58" s="2" t="n">
-        <v>45320</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>45330</v>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>29/01/2024</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>08/02/2024</t>
+        </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -3609,8 +3841,10 @@
       <c r="C59" t="n">
         <v>15</v>
       </c>
-      <c r="D59" s="2" t="n">
-        <v>45306</v>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>15/01/2024</t>
+        </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -3628,8 +3862,10 @@
       <c r="C60" t="n">
         <v>78</v>
       </c>
-      <c r="D60" s="2" t="n">
-        <v>46164</v>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -3647,8 +3883,10 @@
       <c r="C61" t="n">
         <v>95</v>
       </c>
-      <c r="D61" s="2" t="n">
-        <v>45300</v>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>09/01/2024</t>
+        </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -3666,8 +3904,10 @@
       <c r="C62" t="n">
         <v>52</v>
       </c>
-      <c r="D62" s="2" t="n">
-        <v>45298</v>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>07/01/2024</t>
+        </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -3685,8 +3925,10 @@
       <c r="C63" t="n">
         <v>49</v>
       </c>
-      <c r="D63" s="2" t="n">
-        <v>46164</v>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -3704,11 +3946,15 @@
       <c r="C64" t="n">
         <v>67</v>
       </c>
-      <c r="D64" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E64" s="2" t="n">
-        <v>46174</v>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -3726,8 +3972,10 @@
       <c r="C65" t="n">
         <v>27</v>
       </c>
-      <c r="D65" s="2" t="n">
-        <v>45360</v>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>09/03/2024</t>
+        </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -3745,8 +3993,10 @@
       <c r="C66" t="n">
         <v>87</v>
       </c>
-      <c r="D66" s="2" t="n">
-        <v>45360</v>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>09/03/2024</t>
+        </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -3764,11 +4014,15 @@
       <c r="C67" t="n">
         <v>12</v>
       </c>
-      <c r="D67" s="2" t="n">
-        <v>45390</v>
-      </c>
-      <c r="E67" s="2" t="n">
-        <v>45400</v>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>18/04/2024</t>
+        </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -3786,8 +4040,10 @@
       <c r="C68" t="n">
         <v>21</v>
       </c>
-      <c r="D68" s="2" t="n">
-        <v>45382</v>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>31/03/2024</t>
+        </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -3805,11 +4061,15 @@
       <c r="C69" t="n">
         <v>2</v>
       </c>
-      <c r="D69" s="2" t="n">
-        <v>45346</v>
-      </c>
-      <c r="E69" s="2" t="n">
-        <v>45356</v>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>24/02/2024</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>05/03/2024</t>
+        </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -3827,11 +4087,15 @@
       <c r="C70" t="n">
         <v>15</v>
       </c>
-      <c r="D70" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E70" s="2" t="n">
-        <v>46174</v>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -3849,8 +4113,10 @@
       <c r="C71" t="n">
         <v>74</v>
       </c>
-      <c r="D71" s="2" t="n">
-        <v>46164</v>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -3868,11 +4134,15 @@
       <c r="C72" t="n">
         <v>31</v>
       </c>
-      <c r="D72" s="2" t="n">
-        <v>45374</v>
-      </c>
-      <c r="E72" s="2" t="n">
-        <v>45384</v>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>23/03/2024</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>02/04/2024</t>
+        </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -3890,11 +4160,15 @@
       <c r="C73" t="n">
         <v>97</v>
       </c>
-      <c r="D73" s="2" t="n">
-        <v>45374</v>
-      </c>
-      <c r="E73" s="2" t="n">
-        <v>45384</v>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>23/03/2024</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>02/04/2024</t>
+        </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -3912,8 +4186,10 @@
       <c r="C74" t="n">
         <v>79</v>
       </c>
-      <c r="D74" s="2" t="n">
-        <v>45368</v>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>17/03/2024</t>
+        </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -3931,11 +4207,15 @@
       <c r="C75" t="n">
         <v>81</v>
       </c>
-      <c r="D75" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E75" s="2" t="n">
-        <v>46174</v>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -3953,8 +4233,10 @@
       <c r="C76" t="n">
         <v>1</v>
       </c>
-      <c r="D76" s="2" t="n">
-        <v>45390</v>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -3972,8 +4254,10 @@
       <c r="C77" t="n">
         <v>59</v>
       </c>
-      <c r="D77" s="2" t="n">
-        <v>46164</v>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -3991,8 +4275,10 @@
       <c r="C78" t="n">
         <v>82</v>
       </c>
-      <c r="D78" s="2" t="n">
-        <v>45379</v>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>28/03/2024</t>
+        </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -4010,11 +4296,15 @@
       <c r="C79" t="n">
         <v>29</v>
       </c>
-      <c r="D79" s="2" t="n">
-        <v>45348</v>
-      </c>
-      <c r="E79" s="2" t="n">
-        <v>45358</v>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>26/02/2024</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>07/03/2024</t>
+        </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -4032,8 +4322,10 @@
       <c r="C80" t="n">
         <v>33</v>
       </c>
-      <c r="D80" s="2" t="n">
-        <v>46164</v>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -4051,11 +4343,15 @@
       <c r="C81" t="n">
         <v>86</v>
       </c>
-      <c r="D81" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E81" s="2" t="n">
-        <v>46174</v>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -4073,11 +4369,15 @@
       <c r="C82" t="n">
         <v>79</v>
       </c>
-      <c r="D82" s="2" t="n">
-        <v>45385</v>
-      </c>
-      <c r="E82" s="2" t="n">
-        <v>45395</v>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>03/04/2024</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>13/04/2024</t>
+        </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -4095,11 +4395,15 @@
       <c r="C83" t="n">
         <v>20</v>
       </c>
-      <c r="D83" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E83" s="2" t="n">
-        <v>46174</v>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -4117,11 +4421,15 @@
       <c r="C84" t="n">
         <v>11</v>
       </c>
-      <c r="D84" s="2" t="n">
-        <v>45343</v>
-      </c>
-      <c r="E84" s="2" t="n">
-        <v>45353</v>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>21/02/2024</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>02/03/2024</t>
+        </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -4139,11 +4447,15 @@
       <c r="C85" t="n">
         <v>49</v>
       </c>
-      <c r="D85" s="2" t="n">
-        <v>45343</v>
-      </c>
-      <c r="E85" s="2" t="n">
-        <v>45353</v>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>21/02/2024</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>02/03/2024</t>
+        </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -4161,11 +4473,15 @@
       <c r="C86" t="n">
         <v>35</v>
       </c>
-      <c r="D86" s="2" t="n">
-        <v>45376</v>
-      </c>
-      <c r="E86" s="2" t="n">
-        <v>45386</v>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>25/03/2024</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>04/04/2024</t>
+        </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -4183,8 +4499,10 @@
       <c r="C87" t="n">
         <v>60</v>
       </c>
-      <c r="D87" s="2" t="n">
-        <v>45408</v>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>26/04/2024</t>
+        </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -4202,11 +4520,15 @@
       <c r="C88" t="n">
         <v>10</v>
       </c>
-      <c r="D88" s="2" t="n">
-        <v>45373</v>
-      </c>
-      <c r="E88" s="2" t="n">
-        <v>45383</v>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>22/03/2024</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>01/04/2024</t>
+        </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -4224,8 +4546,10 @@
       <c r="C89" t="n">
         <v>73</v>
       </c>
-      <c r="D89" s="2" t="n">
-        <v>45292</v>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>01/01/2024</t>
+        </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -4243,11 +4567,15 @@
       <c r="C90" t="n">
         <v>57</v>
       </c>
-      <c r="D90" s="2" t="n">
-        <v>45349</v>
-      </c>
-      <c r="E90" s="2" t="n">
-        <v>45359</v>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>27/02/2024</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>08/03/2024</t>
+        </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -4265,8 +4593,10 @@
       <c r="C91" t="n">
         <v>28</v>
       </c>
-      <c r="D91" s="2" t="n">
-        <v>45292</v>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>01/01/2024</t>
+        </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -4284,11 +4614,15 @@
       <c r="C92" t="n">
         <v>70</v>
       </c>
-      <c r="D92" s="2" t="n">
-        <v>45296</v>
-      </c>
-      <c r="E92" s="2" t="n">
-        <v>45306</v>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>05/01/2024</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>15/01/2024</t>
+        </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -4306,11 +4640,15 @@
       <c r="C93" t="n">
         <v>78</v>
       </c>
-      <c r="D93" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E93" s="2" t="n">
-        <v>46174</v>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -4328,8 +4666,10 @@
       <c r="C94" t="n">
         <v>64</v>
       </c>
-      <c r="D94" s="2" t="n">
-        <v>45386</v>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>04/04/2024</t>
+        </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -4347,11 +4687,15 @@
       <c r="C95" t="n">
         <v>58</v>
       </c>
-      <c r="D95" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E95" s="2" t="n">
-        <v>46174</v>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -4369,11 +4713,15 @@
       <c r="C96" t="n">
         <v>22</v>
       </c>
-      <c r="D96" s="2" t="n">
-        <v>45321</v>
-      </c>
-      <c r="E96" s="2" t="n">
-        <v>45331</v>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>30/01/2024</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>09/02/2024</t>
+        </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -4391,11 +4739,15 @@
       <c r="C97" t="n">
         <v>11</v>
       </c>
-      <c r="D97" s="2" t="n">
-        <v>45396</v>
-      </c>
-      <c r="E97" s="2" t="n">
-        <v>45406</v>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>14/04/2024</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>24/04/2024</t>
+        </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -4413,11 +4765,15 @@
       <c r="C98" t="n">
         <v>99</v>
       </c>
-      <c r="D98" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E98" s="2" t="n">
-        <v>46174</v>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -4435,11 +4791,15 @@
       <c r="C99" t="n">
         <v>71</v>
       </c>
-      <c r="D99" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E99" s="2" t="n">
-        <v>46174</v>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -4457,8 +4817,10 @@
       <c r="C100" t="n">
         <v>34</v>
       </c>
-      <c r="D100" s="2" t="n">
-        <v>45389</v>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>07/04/2024</t>
+        </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -4476,11 +4838,15 @@
       <c r="C101" t="n">
         <v>30</v>
       </c>
-      <c r="D101" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E101" s="2" t="n">
-        <v>46174</v>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -4498,8 +4864,10 @@
       <c r="C102" t="n">
         <v>59</v>
       </c>
-      <c r="D102" s="2" t="n">
-        <v>45332</v>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>10/02/2024</t>
+        </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -4517,8 +4885,10 @@
       <c r="C103" t="n">
         <v>73</v>
       </c>
-      <c r="D103" s="2" t="n">
-        <v>45308</v>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>17/01/2024</t>
+        </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -4536,8 +4906,10 @@
       <c r="C104" t="n">
         <v>29</v>
       </c>
-      <c r="D104" s="2" t="n">
-        <v>45308</v>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>17/01/2024</t>
+        </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -4555,8 +4927,10 @@
       <c r="C105" t="n">
         <v>70</v>
       </c>
-      <c r="D105" s="2" t="n">
-        <v>45363</v>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>12/03/2024</t>
+        </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -4574,8 +4948,10 @@
       <c r="C106" t="n">
         <v>12</v>
       </c>
-      <c r="D106" s="2" t="n">
-        <v>45320</v>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>29/01/2024</t>
+        </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -4593,8 +4969,10 @@
       <c r="C107" t="n">
         <v>70</v>
       </c>
-      <c r="D107" s="2" t="n">
-        <v>46164</v>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -4612,8 +4990,10 @@
       <c r="C108" t="n">
         <v>12</v>
       </c>
-      <c r="D108" s="2" t="n">
-        <v>45326</v>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>04/02/2024</t>
+        </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -4631,8 +5011,10 @@
       <c r="C109" t="n">
         <v>1</v>
       </c>
-      <c r="D109" s="2" t="n">
-        <v>45304</v>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>13/01/2024</t>
+        </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -4650,11 +5032,15 @@
       <c r="C110" t="n">
         <v>87</v>
       </c>
-      <c r="D110" s="2" t="n">
-        <v>45295</v>
-      </c>
-      <c r="E110" s="2" t="n">
-        <v>45305</v>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>04/01/2024</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>14/01/2024</t>
+        </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -4672,8 +5058,10 @@
       <c r="C111" t="n">
         <v>50</v>
       </c>
-      <c r="D111" s="2" t="n">
-        <v>45379</v>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>28/03/2024</t>
+        </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -4691,11 +5079,15 @@
       <c r="C112" t="n">
         <v>61</v>
       </c>
-      <c r="D112" s="2" t="n">
-        <v>45331</v>
-      </c>
-      <c r="E112" s="2" t="n">
-        <v>45341</v>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>09/02/2024</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>19/02/2024</t>
+        </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -4713,11 +5105,15 @@
       <c r="C113" t="n">
         <v>93</v>
       </c>
-      <c r="D113" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E113" s="2" t="n">
-        <v>46174</v>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -4735,8 +5131,10 @@
       <c r="C114" t="n">
         <v>86</v>
       </c>
-      <c r="D114" s="2" t="n">
-        <v>45330</v>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>08/02/2024</t>
+        </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -4754,8 +5152,10 @@
       <c r="C115" t="n">
         <v>75</v>
       </c>
-      <c r="D115" s="2" t="n">
-        <v>45330</v>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>08/02/2024</t>
+        </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -4773,11 +5173,15 @@
       <c r="C116" t="n">
         <v>9</v>
       </c>
-      <c r="D116" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E116" s="2" t="n">
-        <v>46174</v>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -4795,11 +5199,15 @@
       <c r="C117" t="n">
         <v>50</v>
       </c>
-      <c r="D117" s="2" t="n">
-        <v>45371</v>
-      </c>
-      <c r="E117" s="2" t="n">
-        <v>45381</v>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>20/03/2024</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>30/03/2024</t>
+        </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -4817,11 +5225,15 @@
       <c r="C118" t="n">
         <v>74</v>
       </c>
-      <c r="D118" s="2" t="n">
-        <v>45371</v>
-      </c>
-      <c r="E118" s="2" t="n">
-        <v>45381</v>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>20/03/2024</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>30/03/2024</t>
+        </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -4839,11 +5251,15 @@
       <c r="C119" t="n">
         <v>42</v>
       </c>
-      <c r="D119" s="2" t="n">
-        <v>45371</v>
-      </c>
-      <c r="E119" s="2" t="n">
-        <v>45381</v>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>20/03/2024</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>30/03/2024</t>
+        </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -4861,11 +5277,15 @@
       <c r="C120" t="n">
         <v>63</v>
       </c>
-      <c r="D120" s="2" t="n">
-        <v>45337</v>
-      </c>
-      <c r="E120" s="2" t="n">
-        <v>45347</v>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>15/02/2024</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>25/02/2024</t>
+        </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -4883,11 +5303,15 @@
       <c r="C121" t="n">
         <v>29</v>
       </c>
-      <c r="D121" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E121" s="2" t="n">
-        <v>46174</v>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -4905,8 +5329,10 @@
       <c r="C122" t="n">
         <v>41</v>
       </c>
-      <c r="D122" s="2" t="n">
-        <v>45349</v>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>27/02/2024</t>
+        </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -4924,11 +5350,15 @@
       <c r="C123" t="n">
         <v>43</v>
       </c>
-      <c r="D123" s="2" t="n">
-        <v>45352</v>
-      </c>
-      <c r="E123" s="2" t="n">
-        <v>45362</v>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>01/03/2024</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>11/03/2024</t>
+        </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -4946,8 +5376,10 @@
       <c r="C124" t="n">
         <v>89</v>
       </c>
-      <c r="D124" s="2" t="n">
-        <v>46164</v>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -4965,11 +5397,15 @@
       <c r="C125" t="n">
         <v>60</v>
       </c>
-      <c r="D125" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E125" s="2" t="n">
-        <v>46174</v>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -4987,11 +5423,15 @@
       <c r="C126" t="n">
         <v>21</v>
       </c>
-      <c r="D126" s="2" t="n">
-        <v>45322</v>
-      </c>
-      <c r="E126" s="2" t="n">
-        <v>45332</v>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>31/01/2024</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>10/02/2024</t>
+        </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -5009,8 +5449,10 @@
       <c r="C127" t="n">
         <v>63</v>
       </c>
-      <c r="D127" s="2" t="n">
-        <v>46164</v>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
@@ -5028,8 +5470,10 @@
       <c r="C128" t="n">
         <v>85</v>
       </c>
-      <c r="D128" s="2" t="n">
-        <v>45312</v>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>21/01/2024</t>
+        </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -5047,11 +5491,15 @@
       <c r="C129" t="n">
         <v>82</v>
       </c>
-      <c r="D129" s="2" t="n">
-        <v>45327</v>
-      </c>
-      <c r="E129" s="2" t="n">
-        <v>45337</v>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>05/02/2024</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>15/02/2024</t>
+        </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -5069,11 +5517,15 @@
       <c r="C130" t="n">
         <v>98</v>
       </c>
-      <c r="D130" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E130" s="2" t="n">
-        <v>46174</v>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -5091,11 +5543,15 @@
       <c r="C131" t="n">
         <v>31</v>
       </c>
-      <c r="D131" s="2" t="n">
-        <v>45377</v>
-      </c>
-      <c r="E131" s="2" t="n">
-        <v>45387</v>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>26/03/2024</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>05/04/2024</t>
+        </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -5113,11 +5569,15 @@
       <c r="C132" t="n">
         <v>14</v>
       </c>
-      <c r="D132" s="2" t="n">
-        <v>45359</v>
-      </c>
-      <c r="E132" s="2" t="n">
-        <v>45369</v>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>08/03/2024</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>18/03/2024</t>
+        </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -5135,8 +5595,10 @@
       <c r="C133" t="n">
         <v>15</v>
       </c>
-      <c r="D133" s="2" t="n">
-        <v>45344</v>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>22/02/2024</t>
+        </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -5154,11 +5616,15 @@
       <c r="C134" t="n">
         <v>74</v>
       </c>
-      <c r="D134" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E134" s="2" t="n">
-        <v>46174</v>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -5551,7 +6017,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5604,8 +6070,10 @@
       <c r="E2" t="n">
         <v>4</v>
       </c>
-      <c r="F2" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -5626,8 +6094,10 @@
       <c r="E3" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -5648,8 +6118,10 @@
       <c r="E4" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -5670,8 +6142,10 @@
       <c r="E5" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -5692,8 +6166,10 @@
       <c r="E6" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -5714,8 +6190,10 @@
       <c r="E7" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -5736,8 +6214,10 @@
       <c r="E8" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -5758,8 +6238,10 @@
       <c r="E9" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -5780,8 +6262,10 @@
       <c r="E10" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -5802,8 +6286,10 @@
       <c r="E11" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -5824,8 +6310,10 @@
       <c r="E12" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -5846,8 +6334,10 @@
       <c r="E13" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -5868,8 +6358,10 @@
       <c r="E14" t="n">
         <v>4</v>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -5890,8 +6382,10 @@
       <c r="E15" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -5912,8 +6406,10 @@
       <c r="E16" t="n">
         <v>5</v>
       </c>
-      <c r="F16" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -5934,8 +6430,10 @@
       <c r="E17" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -5956,8 +6454,10 @@
       <c r="E18" t="n">
         <v>5</v>
       </c>
-      <c r="F18" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -5978,8 +6478,10 @@
       <c r="E19" t="n">
         <v>5</v>
       </c>
-      <c r="F19" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -6000,8 +6502,10 @@
       <c r="E20" t="n">
         <v>5</v>
       </c>
-      <c r="F20" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -6022,8 +6526,10 @@
       <c r="E21" t="n">
         <v>3</v>
       </c>
-      <c r="F21" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -6044,8 +6550,10 @@
       <c r="E22" t="n">
         <v>5</v>
       </c>
-      <c r="F22" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -6066,8 +6574,10 @@
       <c r="E23" t="n">
         <v>4</v>
       </c>
-      <c r="F23" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -6088,8 +6598,10 @@
       <c r="E24" t="n">
         <v>5</v>
       </c>
-      <c r="F24" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -6110,8 +6622,10 @@
       <c r="E25" t="n">
         <v>3</v>
       </c>
-      <c r="F25" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -6132,8 +6646,10 @@
       <c r="E26" t="n">
         <v>4</v>
       </c>
-      <c r="F26" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -6154,8 +6670,10 @@
       <c r="E27" t="n">
         <v>5</v>
       </c>
-      <c r="F27" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -6176,8 +6694,10 @@
       <c r="E28" t="n">
         <v>5</v>
       </c>
-      <c r="F28" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -6198,8 +6718,10 @@
       <c r="E29" t="n">
         <v>3</v>
       </c>
-      <c r="F29" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -6220,8 +6742,10 @@
       <c r="E30" t="n">
         <v>5</v>
       </c>
-      <c r="F30" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -6242,8 +6766,10 @@
       <c r="E31" t="n">
         <v>3</v>
       </c>
-      <c r="F31" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -6264,8 +6790,10 @@
       <c r="E32" t="n">
         <v>3</v>
       </c>
-      <c r="F32" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -6286,8 +6814,10 @@
       <c r="E33" t="n">
         <v>3</v>
       </c>
-      <c r="F33" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -6308,8 +6838,10 @@
       <c r="E34" t="n">
         <v>4</v>
       </c>
-      <c r="F34" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -6330,8 +6862,10 @@
       <c r="E35" t="n">
         <v>3</v>
       </c>
-      <c r="F35" s="4" t="n">
-        <v>46164.54162469919</v>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>22/05/2026 13:04:31</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update biblioteca_normalizada.xlsx to reflect recent data changes
</commit_message>
<xml_diff>
--- a/mongo_exports/biblioteca_normalizada.xlsx
+++ b/mongo_exports/biblioteca_normalizada.xlsx
@@ -54,10 +54,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2370,7 +2369,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2399,9 +2398,9 @@
           <t>María García</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>m.garcia@email.com</t>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>3044711957a9f3b4f8210bf6dfc99a5afe6f7f9a52c462522f69f425d3eb5170</t>
         </is>
       </c>
     </row>
@@ -2414,9 +2413,9 @@
           <t>Ana Martínez</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>ana.mar_libros@email.com</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>a738cfbcdbc84a6ae55d630be6c5d269f18b5692264b306f311ac9084f2381e8</t>
         </is>
       </c>
     </row>
@@ -2429,9 +2428,9 @@
           <t>Juan Pérez</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>juan.perez@email.com</t>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3a619cf69213d3aa03721adcee90f43e45fa0443bf1e0d2c11c99f4e7b7792e7</t>
         </is>
       </c>
     </row>
@@ -2444,9 +2443,9 @@
           <t>Carlos López</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>clopez_88@email.com</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>16a87a7917b8083880fdabbc787789432d858a163d71e557ff9db5c77e8dd905</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6071,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6096,7 +6095,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6119,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6143,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6168,7 +6167,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6191,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6215,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6240,7 +6239,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6263,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6287,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6311,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6336,7 +6335,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6360,7 +6359,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6384,7 +6383,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6407,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6431,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6455,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6479,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6504,7 +6503,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6528,7 +6527,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6552,7 +6551,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6576,7 +6575,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6599,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6624,7 +6623,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6648,7 +6647,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6671,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6696,7 +6695,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6720,7 +6719,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6743,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6768,7 +6767,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6791,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6815,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6840,7 +6839,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>
@@ -6864,7 +6863,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>22/05/2026 13:04:31</t>
+          <t>22/05/2026 16:19:34</t>
         </is>
       </c>
     </row>

</xml_diff>